<commit_message>
v2.1.4 (UI): tabla MTBF/MTTR evidencia tesis - fix horas_reparacion_activas + columnas reglas v2.1
</commit_message>
<xml_diff>
--- a/backend/demo_equipos_v21.xlsx
+++ b/backend/demo_equipos_v21.xlsx
@@ -552,7 +552,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -618,7 +618,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -684,7 +684,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -750,7 +750,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -816,7 +816,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -882,7 +882,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -948,7 +948,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1146,7 +1146,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G12" t="inlineStr"/>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -1344,7 +1344,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="G14" t="inlineStr"/>

</xml_diff>